<commit_message>
debugger + uvvenv + explainers excel
</commit_message>
<xml_diff>
--- a/C5_Coursera_Sequence_Models/my_material/explainers_w4_transformer_calculations.xlsx
+++ b/C5_Coursera_Sequence_Models/my_material/explainers_w4_transformer_calculations.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/takis/Documents/sckool/notes-deep-learning/C5_Coursera_Sequence_Models/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/takis/Documents/sckool/notes-deep-learning/C5_Coursera_Sequence_Models/my_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92B276C9-2056-6342-A683-DBAD90A8E173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{140E9928-FA15-DD41-8031-8072176EFA74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="14400" windowHeight="16080" activeTab="1" xr2:uid="{AABB8784-83D0-114F-BA30-ADB4D290B9FE}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16080" activeTab="2" xr2:uid="{AABB8784-83D0-114F-BA30-ADB4D290B9FE}"/>
   </bookViews>
   <sheets>
     <sheet name="attention_calculations" sheetId="1" r:id="rId1"/>
     <sheet name="transformer_calculations" sheetId="2" r:id="rId2"/>
+    <sheet name="cross_attention" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -58,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="87">
   <si>
     <t>the</t>
   </si>
@@ -262,6 +263,63 @@
   </si>
   <si>
     <t>https://levelup.gitconnected.com/understanding-transformers-from-start-to-end-a-step-by-step-math-example-16d4e64e6eb1</t>
+  </si>
+  <si>
+    <t>word</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>d1</t>
+  </si>
+  <si>
+    <t>d2</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=uvEax6XwfJc&amp;list=PLCip3d1iHEMXcAZPhPSb6Br0dykmPKcji&amp;index=14</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>am</t>
+  </si>
+  <si>
+    <t>happy</t>
+  </si>
+  <si>
+    <t>sou</t>
+  </si>
+  <si>
+    <t>feliz</t>
+  </si>
+  <si>
+    <t>input</t>
+  </si>
+  <si>
+    <t>output</t>
+  </si>
+  <si>
+    <t>i</t>
+  </si>
+  <si>
+    <t>Q</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>scale by sqrt(d_model)</t>
+  </si>
+  <si>
+    <t>sou'</t>
+  </si>
+  <si>
+    <t>feliz'</t>
   </si>
 </sst>
 </file>
@@ -302,15 +360,27 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBB6B7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF87A8C4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -318,12 +388,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -362,6 +441,57 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -369,6 +499,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFD1A5D3"/>
+      <color rgb="FF87A8C4"/>
+      <color rgb="FFEBB6B7"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -378,6 +515,1049 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>cross_attention!$B$4:$B$6</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>I</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>am</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>happy</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="38100">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>cross_attention!$D$4:$D$6</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.00</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>-1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.7</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>cross_attention!$E$4:$E$6</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.00</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>-0.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-1.4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-8549-5241-9881-0ACE1D3CA616}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>cross_attention!$B$7:$B$8</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>sou</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>feliz</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:ln w="38100">
+                <a:solidFill>
+                  <a:srgbClr val="C00000"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>cross_attention!$D$7:$D$8</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.00</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>-0.4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.9</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>cross_attention!$E$7:$E$8</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.00</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-8549-5241-9881-0ACE1D3CA616}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>cross_attention!$U$9:$U$10</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>sou'</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>feliz'</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="38100">
+                <a:solidFill>
+                  <a:srgbClr val="D1A5D3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>cross_attention!$V$9:$V$10</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.00</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>-0.65956127914680907</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.59347801063754058</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>cross_attention!$W$9:$W$10</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.00</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>0.48120732053723503</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.86514622748772219</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-8549-5241-9881-0ACE1D3CA616}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="580982832"/>
+        <c:axId val="580984544"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="580982832"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="#,##0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-GR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="580984544"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="580984544"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="#,##0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-GR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="580982832"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-GR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6BFFFFD7-CA3B-6C4E-8B0A-DDDCE10575C1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -857,10 +2037,10 @@
       <c r="O9" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="P9" s="1" t="s">
+      <c r="P9" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="Q9" s="1" t="s">
+      <c r="Q9" s="7" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1197,7 +2377,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="5" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1931,7 +3111,7 @@
       <c r="AI12" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="AJ12" s="11" t="s">
+      <c r="AJ12" s="12" t="s">
         <v>53</v>
       </c>
       <c r="AK12" s="11"/>
@@ -3354,4 +4534,456 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6E9B731-A22B-FF4C-892E-6050CC4F5A8D}">
+  <dimension ref="A1:Z24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="8" width="10.83203125" style="1"/>
+    <col min="9" max="10" width="10.83203125" style="11"/>
+    <col min="11" max="11" width="10.83203125" style="1"/>
+    <col min="12" max="12" width="10.83203125" style="7"/>
+    <col min="13" max="14" width="10.83203125" style="11"/>
+    <col min="15" max="15" width="10.83203125" style="1"/>
+    <col min="16" max="16" width="10.83203125" style="2"/>
+    <col min="17" max="19" width="10.83203125" style="29"/>
+    <col min="20" max="21" width="10.83203125" style="2"/>
+    <col min="22" max="24" width="10.83203125" style="29"/>
+    <col min="25" max="26" width="10.83203125" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="B3" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="P3" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="U3" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="B4" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="D4" s="23">
+        <v>-1</v>
+      </c>
+      <c r="E4" s="23">
+        <v>-0.2</v>
+      </c>
+      <c r="H4" s="7"/>
+      <c r="I4" s="11">
+        <v>1</v>
+      </c>
+      <c r="J4" s="11">
+        <v>0</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="M4" s="11" cm="1">
+        <f t="array" ref="M4:N5">MMULT(D7:E8,I4:J5)</f>
+        <v>-0.4</v>
+      </c>
+      <c r="N4" s="11">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="29" cm="1">
+        <f t="array" ref="Q4:S5">TRANSPOSE(_xlfn.ANCHORARRAY(M9))</f>
+        <v>-1</v>
+      </c>
+      <c r="R4" s="29">
+        <v>-0.7</v>
+      </c>
+      <c r="S4" s="29">
+        <v>1.2</v>
+      </c>
+      <c r="V4" s="29" cm="1">
+        <f t="array" ref="V4:X5">Q23:S24</f>
+        <v>0.29621772031053173</v>
+      </c>
+      <c r="W4" s="29">
+        <v>0.63572752340191541</v>
+      </c>
+      <c r="X4" s="29">
+        <v>6.8054756287552892E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="B5" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="23">
+        <v>-0.7</v>
+      </c>
+      <c r="E5" s="23">
+        <v>1</v>
+      </c>
+      <c r="H5" s="7"/>
+      <c r="I5" s="11">
+        <v>0</v>
+      </c>
+      <c r="J5" s="11">
+        <v>1</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="M5" s="11">
+        <v>0.9</v>
+      </c>
+      <c r="N5" s="11">
+        <v>-0.2</v>
+      </c>
+      <c r="Q5" s="29">
+        <v>-0.2</v>
+      </c>
+      <c r="R5" s="29">
+        <v>1</v>
+      </c>
+      <c r="S5" s="29">
+        <v>-1.4</v>
+      </c>
+      <c r="V5" s="29">
+        <v>0.14647686889885828</v>
+      </c>
+      <c r="W5" s="29">
+        <v>0.14961730409735322</v>
+      </c>
+      <c r="X5" s="29">
+        <v>0.70390582700378845</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="B6" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="D6" s="26">
+        <v>1.2</v>
+      </c>
+      <c r="E6" s="26">
+        <v>-1.4</v>
+      </c>
+      <c r="H6" s="7"/>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="B7" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="D7" s="17">
+        <v>-0.4</v>
+      </c>
+      <c r="E7" s="17">
+        <v>1</v>
+      </c>
+      <c r="H7" s="7"/>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="B8" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" s="20">
+        <v>0.9</v>
+      </c>
+      <c r="E8" s="20">
+        <v>-0.2</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="P8" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="U8" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="V8" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="W8" s="30" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="H9" s="7"/>
+      <c r="I9" s="11">
+        <v>1</v>
+      </c>
+      <c r="J9" s="11">
+        <v>0</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="M9" s="11" cm="1">
+        <f t="array" ref="M9:N11">MMULT(D4:E6,I9:J10)</f>
+        <v>-1</v>
+      </c>
+      <c r="N9" s="11">
+        <v>-0.2</v>
+      </c>
+      <c r="Q9" s="29" cm="1">
+        <f t="array" ref="Q9:S10">MMULT(_xlfn.ANCHORARRAY(M4),_xlfn.ANCHORARRAY(Q4))</f>
+        <v>0.2</v>
+      </c>
+      <c r="R9" s="29">
+        <v>1.28</v>
+      </c>
+      <c r="S9" s="29">
+        <v>-1.88</v>
+      </c>
+      <c r="U9" s="27" t="s">
+        <v>85</v>
+      </c>
+      <c r="V9" s="29" cm="1">
+        <f t="array" ref="V9:W10">MMULT(_xlfn.ANCHORARRAY(V4),_xlfn.ANCHORARRAY(M15))</f>
+        <v>-0.65956127914680907</v>
+      </c>
+      <c r="W9" s="29">
+        <v>0.48120732053723503</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="H10" s="7"/>
+      <c r="I10" s="11">
+        <v>0</v>
+      </c>
+      <c r="J10" s="11">
+        <v>1</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="M10" s="11">
+        <v>-0.7</v>
+      </c>
+      <c r="N10" s="11">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="29">
+        <v>-0.86</v>
+      </c>
+      <c r="R10" s="29">
+        <v>-0.83000000000000007</v>
+      </c>
+      <c r="S10" s="29">
+        <v>1.36</v>
+      </c>
+      <c r="U10" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="V10" s="29">
+        <v>0.59347801063754058</v>
+      </c>
+      <c r="W10" s="29">
+        <v>-0.86514622748772219</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="H11" s="7"/>
+      <c r="L11" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="M11" s="11">
+        <v>1.2</v>
+      </c>
+      <c r="N11" s="11">
+        <v>-1.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="H12" s="7"/>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="H13" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="P13" s="28" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="I14" s="11">
+        <v>1</v>
+      </c>
+      <c r="J14" s="11">
+        <v>0</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="P14" s="29">
+        <f>SQRT(2)</f>
+        <v>1.4142135623730951</v>
+      </c>
+      <c r="Q14" s="29" cm="1">
+        <f t="array" ref="Q14:S15">_xlfn.ANCHORARRAY(Q9)/P14</f>
+        <v>0.1414213562373095</v>
+      </c>
+      <c r="R14" s="29">
+        <v>0.90509667991878073</v>
+      </c>
+      <c r="S14" s="29">
+        <v>-1.3293607486307091</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="I15" s="11">
+        <v>0</v>
+      </c>
+      <c r="J15" s="11">
+        <v>1</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="M15" s="11" cm="1">
+        <f t="array" ref="M15:N17">MMULT(D4:E6,I14:J15)</f>
+        <v>-1</v>
+      </c>
+      <c r="N15" s="11">
+        <v>-0.2</v>
+      </c>
+      <c r="Q15" s="29">
+        <v>-0.60811183182043083</v>
+      </c>
+      <c r="R15" s="29">
+        <v>-0.58689862838483442</v>
+      </c>
+      <c r="S15" s="29">
+        <v>0.96166522241370467</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="L16" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="M16" s="11">
+        <v>-0.7</v>
+      </c>
+      <c r="N16" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="12:19" x14ac:dyDescent="0.2">
+      <c r="L17" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="M17" s="11">
+        <v>1.2</v>
+      </c>
+      <c r="N17" s="11">
+        <v>-1.4</v>
+      </c>
+    </row>
+    <row r="18" spans="12:19" x14ac:dyDescent="0.2">
+      <c r="P18" s="27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="12:19" x14ac:dyDescent="0.2">
+      <c r="P19" s="30">
+        <f>SUM(Q19:S19)</f>
+        <v>3.8887272137579605</v>
+      </c>
+      <c r="Q19" s="29" cm="1">
+        <f t="array" ref="Q19:S20">EXP(_xlfn.ANCHORARRAY(Q14))</f>
+        <v>1.151909910168909</v>
+      </c>
+      <c r="R19" s="29">
+        <v>2.472170920787979</v>
+      </c>
+      <c r="S19" s="29">
+        <v>0.26464638280107261</v>
+      </c>
+    </row>
+    <row r="20" spans="12:19" x14ac:dyDescent="0.2">
+      <c r="P20" s="30">
+        <f>SUM(Q20:S20)</f>
+        <v>3.7164760563880503</v>
+      </c>
+      <c r="Q20" s="29">
+        <v>0.54437777607729831</v>
+      </c>
+      <c r="R20" s="29">
+        <v>0.55604912829914299</v>
+      </c>
+      <c r="S20" s="29">
+        <v>2.6160491520116089</v>
+      </c>
+    </row>
+    <row r="23" spans="12:19" x14ac:dyDescent="0.2">
+      <c r="P23" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q23" s="29" cm="1">
+        <f t="array" ref="Q23:S23">Q19:S19/P19</f>
+        <v>0.29621772031053173</v>
+      </c>
+      <c r="R23" s="29">
+        <v>0.63572752340191541</v>
+      </c>
+      <c r="S23" s="29">
+        <v>6.8054756287552892E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="12:19" x14ac:dyDescent="0.2">
+      <c r="Q24" s="29" cm="1">
+        <f t="array" ref="Q24:S24">Q20:S20/P20</f>
+        <v>0.14647686889885828</v>
+      </c>
+      <c r="R24" s="29">
+        <v>0.14961730409735322</v>
+      </c>
+      <c r="S24" s="29">
+        <v>0.70390582700378845</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>